<commit_message>
Add Georgia RIP data
</commit_message>
<xml_diff>
--- a/dot rip/outputs/DOT_RIP_definitions_scoring_matrices_with_levels.xlsx
+++ b/dot rip/outputs/DOT_RIP_definitions_scoring_matrices_with_levels.xlsx
@@ -88,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -97,6 +97,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -173,6 +176,59 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DefinitionsMatricesLevels" displayName="DefinitionsMatricesLevels" ref="A1:M22" headerRowCount="1">
+  <autoFilter ref="A1:M22"/>
+  <tableColumns count="13">
+    <tableColumn id="1" name="State code"/>
+    <tableColumn id="2" name="State DOT"/>
+    <tableColumn id="3" name="Scoring level / spatial unit"/>
+    <tableColumn id="4" name="Scoring level detail"/>
+    <tableColumn id="5" name="Resilience definition"/>
+    <tableColumn id="6" name="Risk definition / method"/>
+    <tableColumn id="7" name="Criticality definition / method"/>
+    <tableColumn id="8" name="Vulnerability definition / method"/>
+    <tableColumn id="9" name="Risk scoring matrix / formula"/>
+    <tableColumn id="10" name="Criticality scoring matrix"/>
+    <tableColumn id="11" name="Vulnerability scoring matrix"/>
+    <tableColumn id="12" name="Project prioritization scoring matrix"/>
+    <tableColumn id="13" name="Matrix source pages"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ScoringLevels" displayName="ScoringLevels" ref="A1:E22" headerRowCount="1">
+  <autoFilter ref="A1:E22"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="State code"/>
+    <tableColumn id="2" name="State DOT"/>
+    <tableColumn id="3" name="Scoring level / spatial unit"/>
+    <tableColumn id="4" name="Scoring level detail"/>
+    <tableColumn id="5" name="Matrix source pages"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ScoringMatricesLevels" displayName="ScoringMatricesLevels" ref="A1:H22" headerRowCount="1">
+  <autoFilter ref="A1:H22"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="State code"/>
+    <tableColumn id="2" name="State DOT"/>
+    <tableColumn id="3" name="Scoring level / spatial unit"/>
+    <tableColumn id="4" name="Risk scoring matrix / formula"/>
+    <tableColumn id="5" name="Criticality scoring matrix"/>
+    <tableColumn id="6" name="Vulnerability scoring matrix"/>
+    <tableColumn id="7" name="Project prioritization scoring matrix"/>
+    <tableColumn id="8" name="Matrix source pages"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -464,19 +520,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="155" customHeight="1"/>
   <cols>
-    <col width="10.7109375" customWidth="1" min="1" max="1"/>
-    <col width="24.7109375" customWidth="1" min="2" max="2"/>
-    <col width="34.7109375" customWidth="1" min="3" max="3"/>
-    <col width="58.7109375" customWidth="1" min="4" max="4"/>
-    <col width="46.7109375" customWidth="1" min="5" max="5"/>
-    <col width="54.7109375" customWidth="1" min="6" max="8"/>
-    <col width="64.7109375" customWidth="1" min="9" max="9"/>
-    <col width="58.7109375" customWidth="1" min="10" max="10"/>
-    <col width="64.7109375" customWidth="1" min="11" max="12"/>
-    <col width="30.7109375" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="19.8" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="8"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="12"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
+    <col width="24.3" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -547,1340 +606,1407 @@
       </c>
     </row>
     <row r="2" ht="155" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>California / Caltrans</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Asset / project level, not TAZ</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>APR prioritization is for potentially exposed State Highway System assets, including roadways, bridges, and culverts, within Caltrans districts. STCAP/LTCAP selection is project-level. No TAZ-level scoring found.</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>No formal resilience definition found in the downloaded PDF.</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Adaptation Priorities Reports (APRs) rank exposed State Highway System assets using prioritization scores. SCRIPT says scores consider timing of climate impacts, severity/span, asset condition as sensitivity, number of users affected, and network redundancy; district/local knowledge can adjust rankings. STCAP/LTCAP project funding additionally considers recurring damage/failure risk, mobility/economy/safety benefits, community/environment/critical-infrastructure benefits, equity, and secondary GHG/VMT co-benefits. Prioritization scores/rankings; exact numeric scale not disclosed in SCRIPT.</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Used as part of APR prioritization through network redundancy and regional/statewide mobility, economy, goods movement, safety, adjacent communities, environment, and critical infrastructure benefits. No single criticality formula is disclosed in SCRIPT.</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>Vulnerability comes from Caltrans Climate Change Vulnerability Assessments and APRs. APR prioritization adds timing, severity/span, asset condition as sensitivity, users affected, redundancy, and local knowledge.</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>APR prioritization score. Matrix/weights not disclosed in SCRIPT. Factors listed: climate impact timing; severity/span; asset condition as sensitivity; number of system users affected; network redundancy. Scores rank potentially exposed assets.</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>No standalone criticality matrix found. Criticality-like criteria include users affected, redundancy, regional/statewide mobility/economy/goods movement/safety benefits, adjacent communities, environment, critical infrastructure.</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Climate Change Vulnerability Assessments identify exposure to sea level rise, storm surge, cliff retreat, wildfire, precipitation, temperature. APRs add risk metrics on top of vulnerability.</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>STCAP/LTCAP screening: APR or Cal-Adapt vulnerability; recurring damage/failure risk; mobility/economy/safety benefits; community/environment/critical infrastructure benefits; equity; GHG/VMT co-benefits; permitting/policy/schedule alignment.</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>CA pp.29,31-32</t>
         </is>
       </c>
     </row>
     <row r="3" ht="155" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>CO</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Colorado / CDOT</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Enterprise risk + route/asset criticality + project/corridor screening, not TAZ</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>T*C*V risk formula is for CDOT enterprise risks/risk register. Vulnerability/criticality tools apply to transportation assets/routes statewide; 10-Year Plan integration screens project locations against criticality GIS.</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>The State of Colorado defines resilience as ?the ability of communities to rebound, positively adapt to, or thrive amidst changing conditions or challenges?including human-caused and natural disasters?and to maintain quality of life, healthy growth, durable systems, economic vitality, and conservation of resources for present and future generations.?</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>CDOT scores risk as Risk Score = T x C x V. T is threat likelihood/probability, C is consequence of impact, and V is vulnerability/probability that the estimated consequence is realized. Threats and risk scores are updated every four years with the TAMP cycle or as needed. T is scored 1-5; C and V use scoring rubrics referenced in Section 7.1. Product gives risk score.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Criticality reflects the importance of each transportation asset to statewide system operations and resilience. CDOT criticality map uses AADT, redundancy/alternate routes, roadway classification, freight value, social vulnerability index, and tourism value.</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>Vulnerability is the probability that the anticipated consequence of a threat is realized. In CDOT risk formula, V is multiplied with threat likelihood and consequence.</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Risk Score = T x C x V. T = threat likelihood/probability; C = consequences/consideration of risk event; V = vulnerability/probability consequence is realized. T scored 1-5 by frequency/expert judgment; C and V use rubrics referenced in Section 7.1.</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>Criticality map criteria: AADT; redundancy/alternate routes; roadway classification; freight value; social vulnerability index; tourism value. Outputs High/Medium/Low criticality.</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Vulnerability is probability that estimated consequence will be realized; also FHWA-style asset vulnerability considers exposure, likelihood of damage/compromise, and adaptive capacity.</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>10-Year Plan sketch analysis overlays project locations with criticality GIS; high/medium/low criticality used to identify high-opportunity resilience projects.</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>CO pp.15,24-25,41</t>
         </is>
       </c>
     </row>
     <row r="4" ht="155" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>CT</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Connecticut / CTDOT</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Asset level planned, not TAZ</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>CTDOT is developing a VAST-based vulnerability assessment for transportation assets using asset location, condition, characteristics, and surrounding community. No TAZ-level matrix found.</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>The ability to anticipate, prepare for, and adapt to changing conditions and withstand, respond to, and recover rapidly from disruptions.</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>CTDOT is developing a FHWA VAST-based vulnerability assessment. The plan identifies exposure, sensitivity, and adaptive capacity as the indicator types, but Step 4 Assess Vulnerability is still ongoing/refining. No final scoring scale or formula published in the RIP excerpt; VAST-based model under development.</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Criticality is not finalized as a standalone score in the downloaded RIP. CTDOT is developing a VAST-based vulnerability assessment using asset data, surrounding communities, exposure, sensitivity, and adaptive capacity.</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Vulnerability is the predisposition of assets to be adversely affected by natural hazards. CTDOT uses exposure, sensitivity, and adaptive capacity as VAST indicator types; assessment is still being refined.</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>No final risk scoring matrix found. CTDOT states Vulnerability Assessment is ongoing and VAST-based.</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>No final criticality matrix found in downloaded RIP.</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Planned VAST indicator types: exposure, sensitivity, adaptive capacity. Asset data include location, condition, characteristics, surrounding community. Quantitative/qualitative validation ongoing.</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>PROTECT eligible project screening process exists, but no point matrix/weights found in downloaded RIP.</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>CT pp.18-20,58-59</t>
         </is>
       </c>
     </row>
     <row r="5" ht="155" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Delaware / DelDOT</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Roadway segment / bridge-pavement asset / project level, not TAZ</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Frequently flooded roadway matrix scores roadway segments. Quantitative model is for bridge and pavement assets and can be evaluated individually or corridor-wide. Investment strategy is project-level.</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Resilience or resiliency is the ability to anticipate, prepare for, and adapt to changing conditions and withstand, respond to, and recover rapidly from disruptions.</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>DelDOT first used maintenance-district input to identify frequently flooded roadways, then applied a weighted prioritization matrix. It is moving to quantitative annual-risk modeling for bridges and pavement vulnerable to rainfall and sunny-day flooding. Frequently Flooded Roadways matrix: Flood History 50 pts; Flood Data 25 pts; Infrastructure/Traffic 15 pts; Community 10 pts. Subfactors are equally weighted within categories as listed. Quant model outputs risk for assets/corridors.</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Criticality/prioritization factors include evacuation routes, essential facilities, AADT/traffic counts, DTC ridership, community size, employment density, equity, project readiness, bundling, and recent capital work.</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Frequently flooded roadway risk assessment identifies vulnerable flood-prone roadway segments; future quantitative model assesses annual risk for bridge/pavement assets vulnerable to flooding.</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Frequently Flooded Roadways matrix total 100 pts: Flood History 50; Flood Data 25; Infrastructure/Traffic 15; Community 10. Flood History: frequently flooded roadways 50%, UD inundation study 50%. Flood Data: FEMA floodplain 25%, sea level rise 25%, NOAA flood frequency 25%, major river 25%. Infrastructure/Traffic: traffic count 33%, road rating 33%, essential routes 33%. Community: equity focus area, essential facility, community size, employment density, DTC ridership, each 20%.</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Investment criticality factors: evacuation routes; roads serving hospitals/emergency response/evacuation shelters/DelDOT yards; AADT; DTC ridership; community size; employment density.</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Quantitative model under development for annual risk to bridges and pavement vulnerable to rainfall/sunny-day flooding. Factors: owner costs, user costs, probability of threats including embankment erodibility, roadway flooding, bridge flooding, debris potential.</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Prioritized risk ranking is combined with equity, criticality, evacuation needs, redundancy, readiness, bundling, recent work/timeliness, and project-readiness logic checks.</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>DE pp.27-32,41</t>
         </is>
       </c>
     </row>
     <row r="6" ht="155" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Florida / FDOT</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>State Highway System exposure/vulnerability + project-level prioritization, not TAZ</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>FDOT RAP evaluates State Highway System facilities exposed to flooding, storm surge, sea level rise, extreme heat, and wildfire indicators; RAP Data Viewer supports mapped SHS exposure/vulnerability review; Appendix A lists project-level resilience needs and candidate projects.</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>FDOT RAP frames resilience as strengthening the State Highway System so transportation facilities can anticipate, prepare for, adapt to, withstand, respond to, and recover from disruptions from flooding, storms, sea level rise, and other hazards. No single quoted statutory definition was extracted from the RAP text used for this workbook.</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>FDOT RAP uses a statewide vulnerability assessment rather than a single published numeric risk formula. The RAP identifies SHS facilities exposed to resilience stressors and organizes resilience needs through mapped data, district/project review, and project-level prioritization. RAP Data Viewer provides the online map/data interface for reviewing resilience-related SHS layers.</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Criticality is handled through the importance of State Highway System facilities, SIS/strategic corridors, evacuation and mobility functions, district priorities, project readiness, and resilience need context. Appendix A project list includes district, tier, SIS flag, description, time frame, cost, and adaptation strategy.</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>RAP vulnerability assessment focuses on SHS exposure to flooding, storm surge, sea level rise, extreme heat, wildfire, and related resilience stressors. The RAP Data Viewer supports review of mapped vulnerability/exposure layers; results inform resilience needs and project identification.</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>No single public numeric risk score formula found in the RAP. Assessment is based on SHS exposure/vulnerability mapping and resilience need identification, supported by RAP Data Viewer and project screening.</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>No standalone public criticality point matrix found. Criticality-like project attributes include SHS/SIS relevance, district priority, mobility/evacuation function, project readiness, cost, and adaptation strategy in Appendix A.</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>RAP uses mapped exposure/vulnerability layers for SHS facilities; RAP Data Viewer is the public online interface. Specific point weights were not extracted from the public RAP workbook source.</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>Appendix A Project List provides project-level prioritization fields including district, tier, SIS flag, description, time frame, estimated cost, and adaptation strategy. RAP prioritization is project-level, not TAZ-level.</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>FL RAP; RAP Data Viewer; Appendix A Project List</t>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>No scoring level found</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Downloaded file is a Community Engagement Plan; no risk scoring matrix or spatial scoring unit found.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>No formal resilience definition found in the downloaded PDF.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Downloaded FDOT file is a Community Engagement Plan for resilience activities, not the RIP methodology. It discusses identifying vulnerabilities and resilience-related plans/projects but does not define a scoring formula. No scoring scale found in downloaded PDF.</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>No criticality scoring method found in the downloaded Community Engagement Plan.</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>No vulnerability scoring method found in the downloaded Community Engagement Plan.</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>No risk scoring matrix found in downloaded Community Engagement Plan.</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>No criticality scoring matrix found in downloaded Community Engagement Plan.</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>No vulnerability scoring matrix found; document only mentions identifying vulnerabilities generally.</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>No project scoring matrix found in downloaded PDF.</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>FL pp.1-4</t>
         </is>
       </c>
     </row>
     <row r="7" ht="155" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Georgia / GDOT</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Asset level + project screening/prioritization, not TAZ</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>GDOT RIP risk assessment covers pavements, bridges, and culverts statewide. Exposure is developed from county/GDOT district hazard hot spot analysis and hazard-asset pairs; sensitivity uses asset condition; adaptive capacity is assigned at GDOT district level; criticality uses asset and social vulnerability factors. Projects are screened from FY 2024-FY 2034 STIP-X/TIPs/MTPs/Construction Work Program and prioritized at project level.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>The ability to anticipate, prepare for, adapt to changing conditions and withstand, respond, and recover rapidly from disruptions.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Risk is defined as a combination of the likelihood that an asset will experience an extreme event's impact, and the severity or consequence of that impact. Risk can also be defined as the potential for harm expressed as the product of the probability and the consequence of an event and often expressed in relative term as high, moderate, and low. GDOT scores projects based on each asset's dynamic risk, the product of criticality and dynamic vulnerability, determined using an Asset Prioritization Matrix developed by Georgia Tech.</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Criticality: Importance or value of infrastructure asset, in terms of the cost to users, owners, and society from a loss in function. A critical asset is an asset that is so important to a study area that its removal would result in significant losses. The asset criticality score combines GDOT State Route Prioritization Criteria weighted at 80 percent and the CDC/ATSDR Social Vulnerability Index weighted at 20 percent.</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Vulnerability is defined as the degree to which a system is susceptible to, or unable to cope with adverse effects of extreme weather events. In the transportation context, climate vulnerability is a function of the transportation system's exposure to climate effects, sensitivity to climate effects, and adaptive capacity. In MHEVRA, vulnerability is a function of asset exposure, asset sensitivity, and adaptive capacity.</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Dynamic risk = criticality x dynamic vulnerability. GDOT uses the Georgia Tech Asset Prioritization Matrix; project tables classify Criticality Class, Vulnerability Class, Risk Class on a 1-3 scale and Priority as First/Second/Third/Last. Risk results are summarized for pavement, bridges, and culverts.</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Criticality score = 80% GDOT State Route Prioritization Criteria + 20% CDC/ATSDR Social Vulnerability Index. Figure 12 lists factors for estimating criticality score. Project list reports Criticality Class 1-3.</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Vulnerability = asset exposure + asset sensitivity + adaptive capacity within MHEVRA. Exposure uses GIS hot spot analysis of major climate/weather events by county and GDOT district plus hazard-asset pair weights; sensitivity uses Pavement Condition Index, Bridge Sufficiency Rating, and Culvert Condition Index; adaptive capacity uses a resilience rating/scorecard concept with the same unit score assigned to all seven GDOT districts in this assessment. Project list reports Vulnerability Class 1-3.</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Projects between FY 2024 and FY 2034 were screened from STIP-X, STIP, TIPs, MTPs, and the Construction Work Program. Tier 1 maintain/rehabilitate work types receive higher priority; Tier 2 capacity/operational projects need to be on an evacuation route. Further screening uses coastal county, FEMA 1% and 0.2% flood hazard areas, and MHEVRA priority based on criticality/vulnerability/risk where data is available. Table 5 lists recommended projects with Criticality Class, Vulnerability Class, Risk Class, and Priority.</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>GA pp.3-8,26,30-35,39-42,48</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="155" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>IA</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Iowa / Iowa DOT</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Hazard level + project/location level, not TAZ</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Likelihood x consequence scores natural hazards statewide. Project prioritization then ranks submitted resilience projects by criticality of project location and cost effectiveness.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>The Iowa DOT defines resiliency as the ability to anticipate, prepare for, and adapt to changing conditions and withstand, respond to, and quickly recover from disruptions.</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Iowa DOT RWG prioritized natural hazards using a risk-based assessment: risk/vulnerability = likelihood x consequence. Lower likelihood values mean rare events; higher values mean higher probability. Lower consequence values mean lower transportation-system impact; higher values mean significant damage. Hazards grouped into three tiers by risk scores and preferred mitigation approach. Exact numeric scale for likelihood/consequence is shown in matrix/table but not fully extracted as text.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Project-level prioritization ranks projects by how critical the project location is to the system and by cost effectiveness. The exact criticality formula is not published in the extracted RIP text.</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Hazard vulnerability/risk is calculated by multiplying likelihood and consequence. Project screening identifies vulnerabilities and associated hazards before prioritization.</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>Hazard risk/vulnerability = Likelihood x Consequence. Lower likelihood = rare; higher likelihood = higher probability. Lower consequence = lower system impact; higher consequence = significant damage. Hazards grouped into Tier 1/2/3 based on risk scores and preferred mitigation methods.</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>Project prioritization includes how critical the project location is for the system; exact point matrix not disclosed in extracted text.</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Same hazard matrix: likelihood x consequence. Project screening first identifies which vulnerabilities/hazards exist and whether activity is PROTECT eligible.</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>Project selection: annual district solicitation; screening for vulnerabilities and PROTECT eligibility; prioritization by location criticality and cost effectiveness; composite ranking reviewed by RWG and Program Team.</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>IA pp.38-39,53,62</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="155" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9" ht="155" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>KY</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Kentucky / KYTC</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Asset / highway segment level, not TAZ</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>VAST scores transportation assets/highway segments on the NHS by hazard. District results list routes/segments with vulnerability scores; assessment also uses district workshop input.</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Transportation resilience, defined by the Federal Highway Administration (FHWA) as the ability to anticipate, prepare for, and adapt to changing conditions and withstand, respond to, and recover rapidly from disruptions, is an important component of KYTC?s mission.</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>KYTC describes a hybrid risk-based vulnerability assessment: data analysis, district workshops, and GIS compilation. A risk matrix considers likelihood and severity/consequence. Appendix uses FHWA VAST: exposure, sensitivity, and adaptive capacity indicators produce vulnerability scores. Likelihood is 1-5. VAST indicator scores are 1-4; exposure/sensitivity high score = more exposure/sensitivity; adaptive capacity high score = less capacity. Exposure/sensitivity/adaptive capacity default weights are 33% each; final vulnerability score is 1-4, higher = more vulnerable.</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Criticality is treated within VAST adaptive capacity/asset criticality inputs such as AADT, functional class, asset replacement value, and detour route viability.</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>VAST vulnerability score combines exposure, sensitivity, and adaptive capacity. Indicator scores are 1-4; final vulnerability score is 1-4 where higher means more vulnerable.</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Risk matrix considers likelihood and severity/consequence by KYTC district. Likelihood scale 1-5: text shows 1 = Very Likely / occurs repeatedly across wide area, 2 = Likely / occurs more than once to multiple assets, etc. Full matrix in plan section.</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>VAST adaptive capacity/criticality inputs may include AADT, functional class, asset replacement value, detour route viability.</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>FHWA VAST: each indicator score 1-4. Exposure and sensitivity: low score = less exposed/sensitive, high score = more. Adaptive capacity: low score = better adaptive capacity, high score = less. Indicator datasets can be weighted; exposure/sensitivity/adaptive capacity default contribution = 33% each. Output vulnerability score 1-4, higher = higher vulnerability.</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>Assets with vulnerability score &gt;=3.5 are highlighted as high-vulnerability by district/hazard; GIS database supports ranking/maps.</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>KY pp.19,53</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="155" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10" ht="155" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>MD</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Maryland / MDOT</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Hazard rating + modal asset / corridor pilot level, not TAZ</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>MDEM hazard probability is hazard-level statewide. SHA/MDOT vulnerability work is asset-level; US 50/MD 450 pilot reports corridor/asset annual risk costs.</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>No formal resilience definition found in the downloaded PDF.</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>MDOT uses MDEM hazard probability ratings and modal vulnerability assessments. SHA scored roadway assets for threats such as storm surge and sea-level rise. MDOT is moving toward quantitative asset-level risk assessments using asset location, condition/design parameters, and threat likelihood. MDEM hazard probability rating: 1 unlikely (&lt; once/30 years), 2 likely (&lt; once/5 years but &gt; once/30 years), 3 highly likely (&gt; once/5 years). Pilot annual risk cost = owner risk from asset failure/repair + user risk from rerouting.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Criticality appears in MDOT/SHA pilot through system criticality mapping, considering system redundancy, demand, social vulnerability, and other operations-lens factors.</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>MDOT modal vulnerability assessments score assets by threats such as storm surge and sea-level rise. Future quantitative assessments use asset location, condition/design, threat likelihood, and maintenance records.</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Hazard probability matrix from MDEM: 1 = Unlikely, less than once every 30 years; 2 = Likely, less than once every 5 years but more often than once every 30 years; 3 = Highly Likely, more than once every 5 years. Pilot quantitative risk uses annual risk cost = owner risk + user risk.</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>SHA pilot system criticality map considers system redundancy, demand, social vulnerability, and other operations-lens factors. No statewide point matrix in TRIP.</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Modal vulnerability assessments; SHA scored roadway assets for storm surge, sea-level rise, precipitation change. Future model uses asset location, condition, design parameters, threat likelihood, FIRM, maintenance records.</t>
         </is>
       </c>
-      <c r="L9" s="3" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>Prioritization intended to use annualized risk with social/economic/financial impacts; implementation-ready/immediate-benefit projects prioritized for early PROTECT funds.</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>MD pp.11-12,27,29,32</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="155" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11" ht="155" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>MI</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Michigan / MDOT</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Asset level, not TAZ</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Risk score is calculated for assets by hazard: roadway segments, bridges, culverts, pump stations, etc. Results are summarized by asset type and district.</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>No formal resilience definition found in the downloaded PDF.</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>Michigan calculates risk from exposure, sensitivity, and criticality. Formula: Risk = (Criticality Score x 25%) + ((Exposure x 75% + Sensitivity x 25%) x 75%). Vulnerability is the exposure/sensitivity component and contributes 75% of total risk. Each asset score is 1-4. High risk = 3-4; medium = 2-2.99; low = 1-1.99. Exposure and sensitivity tables use percentile/natural-break values and hazard-specific weights.</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>Criticality score is one of three risk components and contributes 25% of total risk. Indicators include AADT, truck AADT, functional class, NHS status, and CEJEST disadvantaged communities.</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Vulnerability is the exposure/sensitivity component of risk: Exposure 75% + Sensitivity 25%, then vulnerability contributes 75% of total risk score.</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>Risk = (Criticality Score x 25%) + (((Exposure x 75%) + (Sensitivity x 25%)) x 75%). Criticality = 25% of overall risk; vulnerability = 75% of overall risk. Within vulnerability, exposure = 75%, sensitivity = 25%.</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>Criticality indicators: AADT, truck AADT, functional class, National Highway System, CEJEST disadvantaged communities. Highest 25th percentile generally scores most critical. Criticality score 1-4.</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>Each asset gets exposure, sensitivity, criticality scores from 1-4. Overall risk categories: High 3-4; Medium 2-2.99; Low 1-1.99. Exposure/sensitivity tables use hazard-specific weights; examples include heat exposure: impervious surface 25%, change in days &gt;90F 25%, heat severity 50%; roadway flood sensitivity: pavement condition good/none=1, fair=2.5, poor=4.</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>High-risk asset counts and factor-level results support project implementation prioritization by asset type and hazard.</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>MI pp.21,24-25,74,80</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="155" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12" ht="155" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>MN</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Minnesota / MnDOT</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Asset / roadway network segment level, not TAZ</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Climate risk scores are assigned to roads, bridges/large culverts, and slopes; project selection is district/ATP project-level. No TAZ scoring found.</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>No formal resilience definition found in the downloaded PDF.</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>MnDOT combines asset-level climate hazard exposure with potential traveler impacts to create climate risk scores for roads, bridges/large culverts, and slopes. Climate risk score categories: Very Low, Low, Medium, High, Very High. Exact numeric calculation not disclosed in main text; Appendix B contains method details.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Traveler impact is a proxy for consequence/criticality, using federal functional classification as a relative estimate of travelers impacted and network density as redundancy/detour proxy.</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Asset-level climate hazard exposure is combined with traveler impacts to produce climate risk scores; hydraulic capacity is not included in the climate risk score.</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Climate risk score = asset-level climate hazard exposure combined with potential traveler impacts. Categories shown as Very Low, Low, Medium, High, Very High. Exact numeric matrix not disclosed in main text.</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>Traveler impacts: federal functional classification as proxy for number of travelers impacted; network density as proxy for redundancy/detour options.</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K12" s="4" t="inlineStr">
         <is>
           <t>Asset hazard exposure across timeframe/emissions scenarios; hydraulic capacity not included in climate risk score. Vulnerability assessment is high-level and planning-oriented.</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>Districts/ATPs select PROTECT Formula projects using RIP guidance and regional priorities; no statewide point matrix disclosed in main text.</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>MN pp.29-30,48,51</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="155" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13" ht="155" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Mississippi / MDOT</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Census tract + asset criticality index, not TAZ</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Vulnerability Index is displayed/scored by census tract. BRIC county data are assigned to census tracts; FEMA NRI and dam hazard scores are also applied to census tracts. Asset Criticality Index then incorporates freight/intermodal network elements.</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Community Vulnerability Definition: The FEMA defines community resilience as a community?s ability to: ? Prepare for anticipated natural hazards ? Adapt to changing conditions ? Withstand and recover rapidly from disruptions.</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Mississippi builds a statewide Vulnerability Index using FEMA NRI and other datasets, plus an Asset Criticality Index. Community vulnerability is scored by inverting BRIC resilience category scores; FEMA NRI hazards use 0-5 risk categories. FEMA NRI: 5 very high, 4 relatively high, 3 relatively moderate, 2 relatively low, 1 very low, 0 no concern/no data. BRIC six categories: upper half = 0, lower half = 1, summed to community vulnerability 1-5. Dam index weights density and hazard class, with high-hazard dams weighted most.</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Asset Criticality Index incorporates the Vulnerability Index, Tier I/Tier II freight networks, and Intermodal Connectors. Detailed full formula not found in selected pages.</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Statewide Vulnerability Index uses FEMA NRI and related datasets. Community vulnerability inverts BRIC resilience categories and sums six category scores; FEMA NRI risks use 0-5 categories.</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>FEMA NRI risk scale used for many hazards: 5 = Very High; 4 = Relatively High; 3 = Relatively Moderate; 2 = Relatively Low; 1 = Very Low; 0 = No Concerns/No Data. Points assigned to census tracts based on NRI.</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>Asset Criticality Index incorporates Vulnerability Index, Tier I/Tier II freight networks, and Intermodal Connectors. Full criticality point matrix not found in selected pages.</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>Community vulnerability BRIC matrix: six BRIC categories each split upper/lower half; upper half/more resilient = 0, lower half/less resilient = 1; sum six category scores. Community Vulnerability Score categories 5 Very High, 4 Relatively High, 3 Relatively Moderate, 2 Relatively Low, 1 Very Low. Dam hazard index: density quartiles scored 1.5/1/0.5/0 plus downstream hazard weighted by class, with high hazard upper half=2, lower half=1, none=0.</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>Vulnerability Index and Asset Criticality Index evaluate/rank system criticality; project matrix not found in selected pages.</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>MS pp.20,26,31,34,37</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="155" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14" ht="155" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>NC</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>North Carolina / NCDOT</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Asset / vulnerable area / STIP project level, not TAZ</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Prioritization scores assets or areas of concern and potential resilience projects that are on the Criticality Map and exposed to hazards. Units include roadways, NBI structures, rail lines, and STIP projects.</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>As defined by the NCDOT Resilience Policy, resiliency is ?the ability to anticipate, prepare for, and adapt to changing conditions and withstand, respond to, and recover rapidly from disruptions?.</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>NCDOT uses a multicriteria resilience prioritization process to rank vulnerable areas/projects using Criticality Score, Exposure Score, and Sensitivity Score. Only assets on the Criticality Map and exposed to selected hazards are scored. Low/Medium/High point process; lowest possible score = 3, highest = 12. Exposure and sensitivity are binned L/M/H; high exposure for two hazards + high sensitivity + high criticality reaches 12.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Criticality Score is one of three prioritization criteria. Only assets/projects on the Criticality Map and exposed to selected hazards are included in scoring.</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Vulnerability/prioritization uses exposure score, sensitivity score, and criticality score. Sensitivity uses pavement IRI, bridge scour/substructure/channel protection, culvert condition, and past washouts.</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Multicriteria point matrix using Criticality Score + Exposure Score + Sensitivity Score. Lowest possible = 3 points; highest possible = 12 points. Only assets/projects on Criticality Map and exposed to selected hazards are scored.</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>Criticality Score from NCDOT Criticality Map; details not fully in extracted pages. Criticality is one of three point components in the 3-12 scoring matrix.</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>Exposure: inland flooding from RIT return intervals (10/25/50/100/500-year), coastal impacts from CRIS/probabilistic SLR, geotechnical from GAM. Sensitivity: roadway IRI &lt;95 good=L, 95-170 fair=M, &gt;170 poor=H; bridges use NBI scour/substructure/channel protection matrices; culverts use NBI Item 62 condition 7-9=L, 5-6=M, 0-4=H; past US-74 washout areas assigned High sensitivity.</t>
         </is>
       </c>
-      <c r="L13" s="3" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>Vulnerable areas and STIP projects on Criticality Map and exposed to hazards are ranked by the 3-12 point score.</t>
         </is>
       </c>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>NC pp.49,51-53</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="155" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="15" ht="155" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>NM</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>New Mexico / NMDOT</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Highway segment / hotspot / project-corridor level, not TAZ</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Resilience risk is assigned to highway segments no more than 1/10 mile long. Segments aggregate into hotspots/corridors; hotspots are ranked statewide and by district.</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Resilience is the ability to avoid, anticipate, absorb, adapt to, and/or rapidly recover from current and future hazards.</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>NMDOT assigns resilience risk to highway segments &lt;=0.1 mile using exposure, sensitivity, and criticality. Scores are converted to High/Medium/Low by percentile and then combined through criticality-specific matrices into A-D risk classes. A = Low, B = Medium, C = High, D = Very High. Exposure/sensitivity/criticality High = 75-100%, Medium = 50-74.9%, Low = 0-49.9%. Hotspot adjusted risk = adjusted exposure score x sensitivity score x criticality score; future exposure adjustment capped at +/-25%.</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Criticality is one of three resilience-risk components. Scores are converted to High/Medium/Low by percentile; any road or structure on the freight network automatically receives High criticality.</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Resilience risk combines exposure, sensitivity, and criticality. These are binned High/Medium/Low by percentile and combined in matrices to A-D risk classes.</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Resilience Risk A-D matrix from Exposure x Sensitivity x Criticality. A=Low, B=Medium, C=High, D=Very High. Exposure/sensitivity/criticality ratings: High=75-100th percentile, Medium=50-74.9th, Low=0-49.9th. Low criticality matrix: high exposure always B; medium exposure A/B/B; low exposure A/A/B. Medium criticality matrix: high exposure B/C/C; medium A/B/C; low A/A/B. High criticality matrix: high exposure C/D/D; medium B/C/D; low B/B/C.</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>Criticality converted to High/Medium/Low by percentile; any road/structure on freight network automatically High criticality.</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>Exposure, sensitivity, criticality are combined into A-D resilience risk. Only assets with some exposure to at least one hazard are scored.</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Hotspots: adjusted exposure for future wildfire/flood/drought, capped at +/-25%; adjusted risk = adjusted exposure x sensitivity x criticality. High/very-high adjacent segments aggregated into corridors; hotspots ranked by length-weighted average adjusted risk.</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="M15" s="4" t="inlineStr">
         <is>
           <t>NM pp.30-32,37</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="155" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16" ht="155" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>OH</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Ohio / ODOT</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Asset level rolled up to corridor/district/state, not TAZ</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Annual risk value is calculated for individual road segments and bridges, then rolled up to corridors, districts, and statewide summaries.</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Resilience is ?the ability to prepare for changing conditions and withstand, respond to, and recover rapidly from disruptions.?</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>ODOT quantifies average annual cost of risk (?risk value?) for flooding, landslides, and rockfalls at asset level, then rolls it up to corridor/district/state scales. Risk value is monetary annualized cost. Example likelihoods include flooding no-damage, flooding damage = flood likelihood x damage likelihood, landslide annual likelihood by susceptibility zone, rockfall likelihood by inventory tier.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>Criticality is reflected indirectly through consequence/user cost, detour length, and staff input on critical sites; future improvements may monetize access to critical services.</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Vulnerability assessment estimates annual closure/damage likelihood and annualized owner/user costs for flooding, landslides, and rockfalls at asset level.</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Annualized risk-cost model. Risk value = average annual cost of risk from threat likelihood/closure probability and consequences. Consequence cost = owner repair/replacement cost + user disruption/detour cost. Example: flooding damage likelihood = flood likelihood x damage likelihood. Landslide likelihood by susceptibility zone; rockfall likelihood by inventory tier.</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr">
         <is>
           <t>Criticality is embedded in user cost, detour length, staff input on critical sites, and potential future valuation of critical services. No separate point matrix found.</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="K16" s="4" t="inlineStr">
         <is>
           <t>Vulnerability assessment covers roads/bridges in/near 100-year floodplain for flooding, landslides, rockfalls. Inputs include closure likelihood, damage duration, repair/replacement assumptions, pavement/bridge condition, landslide susceptibility/history, rockfall inventory.</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="L16" s="4" t="inlineStr">
         <is>
           <t>Priority list developed from risk-based vulnerability assessment results plus district/headquarters input; natural infrastructure/cut sheets for high-vulnerability sites.</t>
         </is>
       </c>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="M16" s="4" t="inlineStr">
         <is>
           <t>OH pp.14,16,27,38,51-52</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="155" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17" ht="155" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>OR</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Oregon / ODOT</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Corridor / highway segment level, not TAZ</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>ODOT scores corridor-scale risk for state highway road segments by hazard and multi-hazard risk. Resilience Corridors are then tiered.</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Resilience is the ability to anticipate, prepare for or adapt to conditions; or withstand, respond to or recover rapidly from system disruptions.</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>ODOT evaluates risk as a function of exposure and consequences. A desktop indicator approach scores exposure and consequence indicators from 1-5 and combines them into corridor-level risk scores by hazard and as multi-hazard risk. Exposure and consequence each 1-5; final risk matrix ranges 1.0-5.0 using average exposure/consequence. Final scores are classified with Jenks natural breaks into low, medium, high, very high.</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Consequences act as the criticality/consequence side of risk, using roadway functional class, AADT traffic flow, and truck AADT flow.</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Risk is assessed from exposure and consequences. Exposure indicators cover nine climate hazards, scored 1-5 and combined with consequences.</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>Quantitative risk matrix: exposure score 1-5 and consequence score 1-5 averaged into risk score 1.0-5.0. Matrix values: if exposure/consequence are 1/1 =&gt; 1.0; 5/5 =&gt; 5.0; each one-point increase in either dimension adds 0.5. Scores classified by Jenks natural breaks into Low, Medium, High, Very High.</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>Consequence measures: functional classification, traffic flow AADT, truck flow AADT. Roadway functional class and AADT indicator scores averaged with equal weights for final consequences score.</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>Exposure to nine hazards scored 1-5: extreme temperature, freeze/thaw, extreme precipitation, snowfall, inland flooding, landslides, wildfire, sea level rise/storm surge, coastal erosion.</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="L17" s="4" t="inlineStr">
         <is>
           <t>Resilience Corridors tiered by future climate, historical hazard events, social disparity status, asset condition, and travel disruption potential; ODOT priority corridors with high truck/traffic flows preferred.</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="M17" s="4" t="inlineStr">
         <is>
           <t>OR pp.58,71,78</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="155" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18" ht="155" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>RI</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Rhode Island / RIDOT</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Asset level + criticality/risk map level, not TAZ</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>VAST vulnerability scores asset classes including roads, bridges, sidewalks, shared-use paths, drainage pipelines, and stormwater treatment units. Criticality/risk maps classify asset locations over time horizons.</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Resilience is defined by RIDOT as the ability of the Rhode Island transportation system to anticipate, prepare for, and adapt to changing conditions; and withstand, respond to, and recover rapidly from any disruptions.</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>RIDOT uses a criticality score, VAST vulnerability assessment, then incorporates risk by combining event likelihood/probability and impacts/consequences with asset vulnerability. Criticality Score = Usage &amp; Operational Importance 60% + Socioeconomic Importance 20% + Health &amp; Safety Importance 20%, then percentile categories High/Medium/Low. VAST asset indicators commonly scored 1-4. Risk/criticality matrix identifies acceptable level of change by year.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>Criticality Score = Usage and Operational Importance 60% + Socioeconomic Importance 20% + Health and Safety Importance 20%; results are classified High/Medium/Low by percentile.</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Vulnerability is assessed using FHWA VAST as a function of exposure, sensitivity, and adaptive capacity. Indicators are scored by asset class, commonly 1-4.</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>Risk assessment incorporates asset vulnerability with likelihood/probability and consequences/impacts of sea-level rise, storm surge, and inland flooding. TAMP uses likelihood x impact matrix; RIP maps criticality/risk by 2035/2050/2100 and checks acceptable level of change.</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>Criticality Score = Usage &amp; Operational Importance 60% + Socioeconomic Importance 20% + Health &amp; Safety Importance 20%. Scores classified High/Medium/Low by percentile.</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>FHWA VAST vulnerability = exposure + sensitivity + adaptive capacity by asset class. Sensitivity example: pavement structural health index 90-100=1, 80-89=2, 70-79=3, 0-69=4. Adaptive capacity examples: low network density scores 4, high density scores 1; downstream stormwater pipes score 4; STU treatment depth 0-2.7 inches scores 4, &gt;7.3 scores 1.</t>
         </is>
       </c>
-      <c r="L17" s="3" t="inlineStr">
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>Need/timeline determined by whether and when risk meets/exceeds acceptable change on criticality/risk matrix maps; project lists and STIP opportunities reviewed.</t>
         </is>
       </c>
-      <c r="M17" s="3" t="inlineStr">
+      <c r="M18" s="4" t="inlineStr">
         <is>
           <t>RI pp.39,44,51,57-58,79,167</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="155" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19" ht="155" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Texas / TxDOT</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Asset level, not TAZ</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Vulnerability is assessed for critical assets by asset type: roadways, bridges/culverts, ITS, maintenance facilities, border crossings, bike/shared-use paths, ports, airports, transit, railways.</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Resilience is the ability to support and maintain a multimodal transportation system that can safely move people, goods, and services during adverse conditions, and to be able to anticipate, prepare for, adapt to, withstand, respond to, and recover efficiently from both human and natural disasters and disruptions.</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>TxDOT?s asset-based vulnerability assessment rates relative vulnerability from minimal to high. Vulnerability combines exposure and sensitivity: exposure is whether assets are in areas subject to disruptors; sensitivity is the degree of damage after exposure. Relative categories minimal-to-high; high vulnerability counts by asset type and district. Numeric scoring formula not published in extracted main-plan text.</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>Evacuation route status is used to prioritize assets for strategy development. The STRP also tracks critical assets and condition/redundancy performance measures, but no numeric criticality formula is published in extracted text.</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Vulnerability is the combination of exposure and sensitivity. Exposure is geospatial overlay of assets with disruptors; sensitivity is the degree to which an asset is damaged after exposure. Results are minimal-to-high.</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Relative vulnerability categories minimal-to-high. Vulnerability = exposure + sensitivity. No numeric risk matrix/formula found in extracted main STRP text.</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
         <is>
           <t>Evacuation route status used to prioritize assets for strategy development. Performance measures track critical assets damaged multiple times, alternate routes, evacuation route condition. No numeric criticality matrix found.</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t>Exposure = geospatial overlay of assets with disruptors. Sensitivity = degree to which asset is damaged after exposure. Results reported as high vulnerability counts by asset type/district/disruptor.</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="L19" s="4" t="inlineStr">
         <is>
           <t>Resilience strategies intended for standard UTP/project selection and funding; cost-benefit analysis may compare resilience investment cost with future disruptor damages for high-cost strategies.</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
+      <c r="M19" s="4" t="inlineStr">
         <is>
           <t>TX pp.57-61,82,85</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="155" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20" ht="155" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>UT</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Utah / UDOT</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Asset segment + candidate project level, not TAZ</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Exposure/criticality risk is calculated for asset segments. Candidate projects receive risk scores by spatial overlay, using maximum segment risk and length-weighted average segment risk.</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>FHWA defines resilience as the ability to anticipate, prepare for, or adapt to conditions or withstand, respond to, or recover rapidly from disruptions.</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>UDOT combines normalized exposure and criticality into resilience risk, then combines candidate-project resilience risk with project efficacy scoring for PROTECT prioritization. Criticality criteria normalized 1-4 and summed equally. Resilience risk combines exposure and criticality and is converted to Low Risk through Very High Risk using Jenks natural breaks. Candidate project risk uses length-weighted average asset-segment risk as preferred basis; project efficacy normalized 1-100; combined score = (project resilience risk + normalized project efficacy) / 2 with equal weights.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Criticality criteria are normalized 1-4 and summed equally: system redundancy, AADT, truck AADT, disadvantaged community index, proximity to community assets, and transit/bike service.</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>Resilience risk combines normalized exposure and criticality. Project risk is assigned using max segment risk and length-weighted average segment risk; length-weighted average is used for prioritization.</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>Resilience risk combines normalized exposure score and normalized criticality score. Both use same scale/max and contribute equally. Final risk categories Low to Very High using Jenks natural breaks.</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
         <is>
           <t>Criticality criteria normalized 1-4: system redundancy, AADT, truck AADT, disadvantaged community index, proximity to community assets, transit/bike service. All criteria contribute equally and are summed to criticality score.</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="K20" s="4" t="inlineStr">
         <is>
           <t>No separate sensitivity/adaptive capacity component in the extracted UDOT risk equation; asset resilience risk is exposure + criticality.</t>
         </is>
       </c>
-      <c r="L19" s="3" t="inlineStr">
+      <c r="L20" s="4" t="inlineStr">
         <is>
           <t>Candidate project risk assigned two ways: maximum overlapping asset-segment risk and length-weighted average of segment risk. Length-weighted average is basis for prioritized list. Project efficacy score normalized 1-100. Combined score = (candidate project resilience risk + normalized project efficacy score) / 2, equal weights.</t>
         </is>
       </c>
-      <c r="M19" s="3" t="inlineStr">
+      <c r="M20" s="4" t="inlineStr">
         <is>
           <t>UT pp.52,56,59-60</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="155" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21" ht="155" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>VA</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Virginia / VDOT</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Asset/infrastructure level planned, not TAZ</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>VDOT framework is for infrastructure assets/new construction/existing infrastructure. Planned scoring uses exposure, sensitivity, and criticality for assets; no final TAZ-level matrix.</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>For the purposes of this plan, resilience is the capability of a transportation project or strategy to anticipate, prepare for, respond to, or recover from significant multi hazard threats with minimum damage and disruption to the transportation network.</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>VDOT plans a risk-based screening approach using exposure, sensitivity, and criticality. Overall vulnerability will be determined by assigning weights/percentages to those three elements. No final weights or numeric scoring scale published in the downloaded plan; methodology is to be developed and integrated into business practices.</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>Planned criticality criteria include AADT, roadway designation, redundancy, primary evacuation route status, and important infrastructure; weights are not finalized in the downloaded plan.</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>Overall vulnerability will be calculated by assigning weights to exposure, sensitivity, and criticality; weights and scoring scale are not finalized in the downloaded plan.</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>Framework planned, no final matrix. Overall vulnerability will be calculated by assigning weights/percentages to exposure, sensitivity, and criticality.</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
         <is>
           <t>Planned criteria: AADT, roadway designation, redundancy, primary evacuation route, important infrastructure. Weights not finalized.</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K21" s="4" t="inlineStr">
         <is>
           <t>Planned elements: exposure to SLR/storm surge/inland flooding and other hazards; sensitivity based on asset condition; criticality. Overall vulnerability = weighted combination of those three elements, but weights not published.</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
+      <c r="L21" s="4" t="inlineStr">
         <is>
           <t>Resilience measures can be evaluated through multi-criteria analysis. Steering Committee selects criteria, weights, and ratings; can eliminate measures that do not score well on important criteria. Cost-effectiveness analysis also used.</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="M21" s="4" t="inlineStr">
         <is>
           <t>VA pp.25-26,48,55</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="155" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>VT</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Vermont / VTrans</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Project screening level, not TAZ</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Draft prioritization is a project idea screening table with Yes=1 flags for vulnerable/critical/in-design/ready-to-build locations. No asset or TAZ formula found.</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>No formal resilience definition found in the downloaded PDF.</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>Downloaded VTrans file is a RIP process slide deck. It proposes screening potential projects with yes/no measures and a draft prioritization scan. Draft prioritization uses Yes=1 for listed flags and sums them. No asset-level risk scoring formula found.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>Draft screening asks whether a project increases redundancy for Functional Class 1, 2, and 3 roads, transit, or rail, and whether it improves freight access. No full criticality formula found.</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>Draft prioritization uses yes/no flags for high-risk or documented repeat-damage locations and highly vulnerable/highly critical locations. No asset vulnerability formula found.</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>Draft screening only. Yes/No flags summed: Highly Vulnerable Location Yes=1; Highly Critical Location Yes=1; Project In Design Yes=1; Ready To Build Yes=1. No full risk matrix found.</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr">
         <is>
           <t>Draft screening asks whether project backs up/increases redundancy for Functional Class 1, 2, and 3 roads, transit, or rail; and whether it improves freight access. Highly Critical Location flag Yes=1.</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="K22" s="4" t="inlineStr">
         <is>
           <t>Draft screening asks if project makes a high-risk or documented repeat damage location less likely to be damaged. Highly Vulnerable Location flag Yes=1.</t>
         </is>
       </c>
-      <c r="L21" s="3" t="inlineStr">
+      <c r="L22" s="4" t="inlineStr">
         <is>
           <t>Draft prioritization scan uses TRPT and Capital Program contents; likely coordinated with VPSP2; yes flags summed for priority scan.</t>
         </is>
       </c>
-      <c r="M21" s="3" t="inlineStr">
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>VT pp.2-4,9-10</t>
         </is>
@@ -1889,6 +2015,9 @@
   </sheetData>
   <autoFilter ref="A1:M21"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1898,14 +2027,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="120" customHeight="1"/>
   <cols>
-    <col width="10.7109375" customWidth="1" min="1" max="1"/>
-    <col width="24.7109375" customWidth="1" min="2" max="2"/>
-    <col width="36.7109375" customWidth="1" min="3" max="3"/>
-    <col width="80.7109375" customWidth="1" min="4" max="4"/>
-    <col width="30.7109375" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="19.8" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="24.3" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1936,540 +2065,567 @@
       </c>
     </row>
     <row r="2" ht="120" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>California / Caltrans</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Asset / project level, not TAZ</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>APR prioritization is for potentially exposed State Highway System assets, including roadways, bridges, and culverts, within Caltrans districts. STCAP/LTCAP selection is project-level. No TAZ-level scoring found.</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>CA pp.29,31-32</t>
         </is>
       </c>
     </row>
     <row r="3" ht="120" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>CO</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Colorado / CDOT</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Enterprise risk + route/asset criticality + project/corridor screening, not TAZ</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>T*C*V risk formula is for CDOT enterprise risks/risk register. Vulnerability/criticality tools apply to transportation assets/routes statewide; 10-Year Plan integration screens project locations against criticality GIS.</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>CO pp.15,24-25,41</t>
         </is>
       </c>
     </row>
     <row r="4" ht="120" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>CT</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Connecticut / CTDOT</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Asset level planned, not TAZ</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>CTDOT is developing a VAST-based vulnerability assessment for transportation assets using asset location, condition, characteristics, and surrounding community. No TAZ-level matrix found.</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>CT pp.18-20,58-59</t>
         </is>
       </c>
     </row>
     <row r="5" ht="120" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Delaware / DelDOT</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Roadway segment / bridge-pavement asset / project level, not TAZ</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Frequently flooded roadway matrix scores roadway segments. Quantitative model is for bridge and pavement assets and can be evaluated individually or corridor-wide. Investment strategy is project-level.</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>DE pp.27-32,41</t>
         </is>
       </c>
     </row>
     <row r="6" ht="120" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Florida / FDOT</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>State Highway System exposure/vulnerability + project-level prioritization, not TAZ</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>FDOT RAP evaluates SHS exposure/vulnerability through mapped data and identifies project-level resilience needs in Appendix A. RAP Data Viewer supports online map/data review.</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>FL RAP; RAP Data Viewer; Appendix A Project List</t>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>No scoring level found</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Downloaded file is a Community Engagement Plan; no risk scoring matrix or spatial scoring unit found.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>FL pp.1-4</t>
         </is>
       </c>
     </row>
     <row r="7" ht="120" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Georgia / GDOT</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Asset level + project screening/prioritization, not TAZ</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>GDOT RIP risk assessment covers pavements, bridges, and culverts statewide. Exposure is developed from county/GDOT district hazard hot spot analysis and hazard-asset pairs; sensitivity uses asset condition; adaptive capacity is assigned at GDOT district level; criticality uses asset and social vulnerability factors. Projects are screened from FY 2024-FY 2034 STIP-X/TIPs/MTPs/Construction Work Program and prioritized at project level.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>GA pp.3-8,26,30-35,39-42,48</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="120" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>IA</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Iowa / Iowa DOT</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Hazard level + project/location level, not TAZ</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Likelihood x consequence scores natural hazards statewide. Project prioritization then ranks submitted resilience projects by criticality of project location and cost effectiveness.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>IA pp.38-39,53,62</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="120" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9" ht="120" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>KY</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Kentucky / KYTC</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Asset / highway segment level, not TAZ</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>VAST scores transportation assets/highway segments on the NHS by hazard. District results list routes/segments with vulnerability scores; assessment also uses district workshop input.</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>KY pp.19,53</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="120" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10" ht="120" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>MD</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Maryland / MDOT</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Hazard rating + modal asset / corridor pilot level, not TAZ</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>MDEM hazard probability is hazard-level statewide. SHA/MDOT vulnerability work is asset-level; US 50/MD 450 pilot reports corridor/asset annual risk costs.</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>MD pp.11-12,27,29,32</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="120" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11" ht="120" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>MI</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Michigan / MDOT</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Asset level, not TAZ</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Risk score is calculated for assets by hazard: roadway segments, bridges, culverts, pump stations, etc. Results are summarized by asset type and district.</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>MI pp.21,24-25,74,80</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="120" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12" ht="120" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>MN</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Minnesota / MnDOT</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Asset / roadway network segment level, not TAZ</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Climate risk scores are assigned to roads, bridges/large culverts, and slopes; project selection is district/ATP project-level. No TAZ scoring found.</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>MN pp.29-30,48,51</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="120" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13" ht="120" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Mississippi / MDOT</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Census tract + asset criticality index, not TAZ</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Vulnerability Index is displayed/scored by census tract. BRIC county data are assigned to census tracts; FEMA NRI and dam hazard scores are also applied to census tracts. Asset Criticality Index then incorporates freight/intermodal network elements.</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>MS pp.20,26,31,34,37</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="120" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14" ht="120" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>NC</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>North Carolina / NCDOT</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Asset / vulnerable area / STIP project level, not TAZ</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Prioritization scores assets or areas of concern and potential resilience projects that are on the Criticality Map and exposed to hazards. Units include roadways, NBI structures, rail lines, and STIP projects.</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>NC pp.49,51-53</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="120" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="15" ht="120" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>NM</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>New Mexico / NMDOT</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Highway segment / hotspot / project-corridor level, not TAZ</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Resilience risk is assigned to highway segments no more than 1/10 mile long. Segments aggregate into hotspots/corridors; hotspots are ranked statewide and by district.</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>NM pp.30-32,37</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="120" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16" ht="120" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>OH</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Ohio / ODOT</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Asset level rolled up to corridor/district/state, not TAZ</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Annual risk value is calculated for individual road segments and bridges, then rolled up to corridors, districts, and statewide summaries.</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>OH pp.14,16,27,38,51-52</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="120" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>OR</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Oregon / ODOT</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Corridor / highway segment level, not TAZ</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>ODOT scores corridor-scale risk for state highway road segments by hazard and multi-hazard risk. Resilience Corridors are then tiered.</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>OR pp.58,71,78</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="120" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18" ht="120" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>RI</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Rhode Island / RIDOT</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Asset level + criticality/risk map level, not TAZ</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>VAST vulnerability scores asset classes including roads, bridges, sidewalks, shared-use paths, drainage pipelines, and stormwater treatment units. Criticality/risk maps classify asset locations over time horizons.</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>RI pp.39,44,51,57-58,79,167</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="120" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19" ht="120" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Texas / TxDOT</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Asset level, not TAZ</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Vulnerability is assessed for critical assets by asset type: roadways, bridges/culverts, ITS, maintenance facilities, border crossings, bike/shared-use paths, ports, airports, transit, railways.</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>TX pp.57-61,82,85</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="120" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20" ht="120" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>UT</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Utah / UDOT</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Asset segment + candidate project level, not TAZ</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Exposure/criticality risk is calculated for asset segments. Candidate projects receive risk scores by spatial overlay, using maximum segment risk and length-weighted average segment risk.</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>UT pp.52,56,59-60</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="120" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21" ht="120" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>VA</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Virginia / VDOT</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Asset/infrastructure level planned, not TAZ</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>VDOT framework is for infrastructure assets/new construction/existing infrastructure. Planned scoring uses exposure, sensitivity, and criticality for assets; no final TAZ-level matrix.</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>VA pp.25-26,48,55</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="120" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>VT</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Vermont / VTrans</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Project screening level, not TAZ</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Draft prioritization is a project idea screening table with Yes=1 flags for vulnerable/critical/in-design/ready-to-build locations. No asset or TAZ formula found.</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>VT pp.2-4,9-10</t>
         </is>
@@ -2478,6 +2634,9 @@
   </sheetData>
   <autoFilter ref="A1:E21"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -2487,16 +2646,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="170" customHeight="1"/>
   <cols>
-    <col width="10.7109375" customWidth="1" min="1" max="1"/>
-    <col width="24.7109375" customWidth="1" min="2" max="2"/>
-    <col width="36.7109375" customWidth="1" min="3" max="3"/>
-    <col width="70.7109375" customWidth="1" min="4" max="4"/>
-    <col width="62.7109375" customWidth="1" min="5" max="5"/>
-    <col width="70.7109375" customWidth="1" min="6" max="7"/>
-    <col width="30.7109375" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="19.8" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="24.3" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2542,840 +2702,882 @@
       </c>
     </row>
     <row r="2" ht="170" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>California / Caltrans</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Asset / project level, not TAZ</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>APR prioritization score. Matrix/weights not disclosed in SCRIPT. Factors listed: climate impact timing; severity/span; asset condition as sensitivity; number of system users affected; network redundancy. Scores rank potentially exposed assets.</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>No standalone criticality matrix found. Criticality-like criteria include users affected, redundancy, regional/statewide mobility/economy/goods movement/safety benefits, adjacent communities, environment, critical infrastructure.</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Climate Change Vulnerability Assessments identify exposure to sea level rise, storm surge, cliff retreat, wildfire, precipitation, temperature. APRs add risk metrics on top of vulnerability.</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>STCAP/LTCAP screening: APR or Cal-Adapt vulnerability; recurring damage/failure risk; mobility/economy/safety benefits; community/environment/critical infrastructure benefits; equity; GHG/VMT co-benefits; permitting/policy/schedule alignment.</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>CA pp.29,31-32</t>
         </is>
       </c>
     </row>
     <row r="3" ht="170" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>CO</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Colorado / CDOT</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Enterprise risk + route/asset criticality + project/corridor screening, not TAZ</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Risk Score = T x C x V. T = threat likelihood/probability; C = consequences/consideration of risk event; V = vulnerability/probability consequence is realized. T scored 1-5 by frequency/expert judgment; C and V use rubrics referenced in Section 7.1.</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Criticality map criteria: AADT; redundancy/alternate routes; roadway classification; freight value; social vulnerability index; tourism value. Outputs High/Medium/Low criticality.</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Vulnerability is probability that estimated consequence will be realized; also FHWA-style asset vulnerability considers exposure, likelihood of damage/compromise, and adaptive capacity.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>10-Year Plan sketch analysis overlays project locations with criticality GIS; high/medium/low criticality used to identify high-opportunity resilience projects.</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>CO pp.15,24-25,41</t>
         </is>
       </c>
     </row>
     <row r="4" ht="170" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>CT</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Connecticut / CTDOT</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Asset level planned, not TAZ</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>No final risk scoring matrix found. CTDOT states Vulnerability Assessment is ongoing and VAST-based.</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>No final criticality matrix found in downloaded RIP.</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Planned VAST indicator types: exposure, sensitivity, adaptive capacity. Asset data include location, condition, characteristics, surrounding community. Quantitative/qualitative validation ongoing.</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>PROTECT eligible project screening process exists, but no point matrix/weights found in downloaded RIP.</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>CT pp.18-20,58-59</t>
         </is>
       </c>
     </row>
     <row r="5" ht="170" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Delaware / DelDOT</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Roadway segment / bridge-pavement asset / project level, not TAZ</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Frequently Flooded Roadways matrix total 100 pts: Flood History 50; Flood Data 25; Infrastructure/Traffic 15; Community 10. Flood History: frequently flooded roadways 50%, UD inundation study 50%. Flood Data: FEMA floodplain 25%, sea level rise 25%, NOAA flood frequency 25%, major river 25%. Infrastructure/Traffic: traffic count 33%, road rating 33%, essential routes 33%. Community: equity focus area, essential facility, community size, employment density, DTC ridership, each 20%.</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Investment criticality factors: evacuation routes; roads serving hospitals/emergency response/evacuation shelters/DelDOT yards; AADT; DTC ridership; community size; employment density.</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Quantitative model under development for annual risk to bridges and pavement vulnerable to rainfall/sunny-day flooding. Factors: owner costs, user costs, probability of threats including embankment erodibility, roadway flooding, bridge flooding, debris potential.</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Prioritized risk ranking is combined with equity, criticality, evacuation needs, redundancy, readiness, bundling, recent work/timeliness, and project-readiness logic checks.</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>DE pp.27-32,41</t>
         </is>
       </c>
     </row>
     <row r="6" ht="170" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Florida / FDOT</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>State Highway System exposure/vulnerability + project-level prioritization, not TAZ</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>No single public numeric risk score formula found in RAP. Assessment uses SHS exposure/vulnerability mapping, resilience need identification, RAP Data Viewer, and project-level screening.</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>No standalone public criticality point matrix found. Criticality-like attributes include SHS/SIS relevance, district priority, mobility/evacuation function, project readiness, cost, and adaptation strategy in Appendix A.</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>RAP uses mapped exposure/vulnerability layers for SHS facilities; RAP Data Viewer is the public online interface. Specific point weights were not extracted from the public RAP workbook source.</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Appendix A Project List provides project-level prioritization fields including district, tier, SIS flag, description, time frame, estimated cost, and adaptation strategy. RAP prioritization is project-level, not TAZ-level.</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>FL RAP; RAP Data Viewer; Appendix A Project List</t>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>No scoring level found</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>No risk scoring matrix found in downloaded Community Engagement Plan.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>No criticality scoring matrix found in downloaded Community Engagement Plan.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>No vulnerability scoring matrix found; document only mentions identifying vulnerabilities generally.</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>No project scoring matrix found in downloaded PDF.</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>FL pp.1-4</t>
         </is>
       </c>
     </row>
     <row r="7" ht="170" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Georgia / GDOT</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Asset level + project screening/prioritization, not TAZ</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Dynamic risk = criticality x dynamic vulnerability. GDOT uses the Georgia Tech Asset Prioritization Matrix; project tables classify Criticality Class, Vulnerability Class, Risk Class on a 1-3 scale and Priority as First/Second/Third/Last. Risk results are summarized for pavement, bridges, and culverts.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Criticality score = 80% GDOT State Route Prioritization Criteria + 20% CDC/ATSDR Social Vulnerability Index. Figure 12 lists factors for estimating criticality score. Project list reports Criticality Class 1-3.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Vulnerability = asset exposure + asset sensitivity + adaptive capacity within MHEVRA. Exposure uses GIS hot spot analysis of major climate/weather events by county and GDOT district plus hazard-asset pair weights; sensitivity uses Pavement Condition Index, Bridge Sufficiency Rating, and Culvert Condition Index; adaptive capacity uses a resilience rating/scorecard concept with the same unit score assigned to all seven GDOT districts in this assessment. Project list reports Vulnerability Class 1-3.</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Projects between FY 2024 and FY 2034 were screened from STIP-X, STIP, TIPs, MTPs, and the Construction Work Program. Tier 1 maintain/rehabilitate work types receive higher priority; Tier 2 capacity/operational projects need to be on an evacuation route. Further screening uses coastal county, FEMA 1% and 0.2% flood hazard areas, and MHEVRA priority based on criticality/vulnerability/risk where data is available. Table 5 lists recommended projects with Criticality Class, Vulnerability Class, Risk Class, and Priority.</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>GA pp.3-8,26,30-35,39-42,48</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="170" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>IA</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Iowa / Iowa DOT</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Hazard level + project/location level, not TAZ</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Hazard risk/vulnerability = Likelihood x Consequence. Lower likelihood = rare; higher likelihood = higher probability. Lower consequence = lower system impact; higher consequence = significant damage. Hazards grouped into Tier 1/2/3 based on risk scores and preferred mitigation methods.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Project prioritization includes how critical the project location is for the system; exact point matrix not disclosed in extracted text.</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Same hazard matrix: likelihood x consequence. Project screening first identifies which vulnerabilities/hazards exist and whether activity is PROTECT eligible.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Project selection: annual district solicitation; screening for vulnerabilities and PROTECT eligibility; prioritization by location criticality and cost effectiveness; composite ranking reviewed by RWG and Program Team.</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>IA pp.38-39,53,62</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="170" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9" ht="170" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>KY</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Kentucky / KYTC</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Asset / highway segment level, not TAZ</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Risk matrix considers likelihood and severity/consequence by KYTC district. Likelihood scale 1-5: text shows 1 = Very Likely / occurs repeatedly across wide area, 2 = Likely / occurs more than once to multiple assets, etc. Full matrix in plan section.</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>VAST adaptive capacity/criticality inputs may include AADT, functional class, asset replacement value, detour route viability.</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>FHWA VAST: each indicator score 1-4. Exposure and sensitivity: low score = less exposed/sensitive, high score = more. Adaptive capacity: low score = better adaptive capacity, high score = less. Indicator datasets can be weighted; exposure/sensitivity/adaptive capacity default contribution = 33% each. Output vulnerability score 1-4, higher = higher vulnerability.</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Assets with vulnerability score &gt;=3.5 are highlighted as high-vulnerability by district/hazard; GIS database supports ranking/maps.</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>KY pp.19,53</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="170" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10" ht="170" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>MD</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Maryland / MDOT</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Hazard rating + modal asset / corridor pilot level, not TAZ</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Hazard probability matrix from MDEM: 1 = Unlikely, less than once every 30 years; 2 = Likely, less than once every 5 years but more often than once every 30 years; 3 = Highly Likely, more than once every 5 years. Pilot quantitative risk uses annual risk cost = owner risk + user risk.</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>SHA pilot system criticality map considers system redundancy, demand, social vulnerability, and other operations-lens factors. No statewide point matrix in TRIP.</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Modal vulnerability assessments; SHA scored roadway assets for storm surge, sea-level rise, precipitation change. Future model uses asset location, condition, design parameters, threat likelihood, FIRM, maintenance records.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Prioritization intended to use annualized risk with social/economic/financial impacts; implementation-ready/immediate-benefit projects prioritized for early PROTECT funds.</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>MD pp.11-12,27,29,32</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="170" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11" ht="170" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>MI</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Michigan / MDOT</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Asset level, not TAZ</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Risk = (Criticality Score x 25%) + (((Exposure x 75%) + (Sensitivity x 25%)) x 75%). Criticality = 25% of overall risk; vulnerability = 75% of overall risk. Within vulnerability, exposure = 75%, sensitivity = 25%.</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Criticality indicators: AADT, truck AADT, functional class, National Highway System, CEJEST disadvantaged communities. Highest 25th percentile generally scores most critical. Criticality score 1-4.</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>Each asset gets exposure, sensitivity, criticality scores from 1-4. Overall risk categories: High 3-4; Medium 2-2.99; Low 1-1.99. Exposure/sensitivity tables use hazard-specific weights; examples include heat exposure: impervious surface 25%, change in days &gt;90F 25%, heat severity 50%; roadway flood sensitivity: pavement condition good/none=1, fair=2.5, poor=4.</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>High-risk asset counts and factor-level results support project implementation prioritization by asset type and hazard.</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>MI pp.21,24-25,74,80</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="170" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12" ht="170" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>MN</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Minnesota / MnDOT</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Asset / roadway network segment level, not TAZ</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Climate risk score = asset-level climate hazard exposure combined with potential traveler impacts. Categories shown as Very Low, Low, Medium, High, Very High. Exact numeric matrix not disclosed in main text.</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Traveler impacts: federal functional classification as proxy for number of travelers impacted; network density as proxy for redundancy/detour options.</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Asset hazard exposure across timeframe/emissions scenarios; hydraulic capacity not included in climate risk score. Vulnerability assessment is high-level and planning-oriented.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Districts/ATPs select PROTECT Formula projects using RIP guidance and regional priorities; no statewide point matrix disclosed in main text.</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>MN pp.29-30,48,51</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="170" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13" ht="170" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Mississippi / MDOT</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Census tract + asset criticality index, not TAZ</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>FEMA NRI risk scale used for many hazards: 5 = Very High; 4 = Relatively High; 3 = Relatively Moderate; 2 = Relatively Low; 1 = Very Low; 0 = No Concerns/No Data. Points assigned to census tracts based on NRI.</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Asset Criticality Index incorporates Vulnerability Index, Tier I/Tier II freight networks, and Intermodal Connectors. Full criticality point matrix not found in selected pages.</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Community vulnerability BRIC matrix: six BRIC categories each split upper/lower half; upper half/more resilient = 0, lower half/less resilient = 1; sum six category scores. Community Vulnerability Score categories 5 Very High, 4 Relatively High, 3 Relatively Moderate, 2 Relatively Low, 1 Very Low. Dam hazard index: density quartiles scored 1.5/1/0.5/0 plus downstream hazard weighted by class, with high hazard upper half=2, lower half=1, none=0.</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Vulnerability Index and Asset Criticality Index evaluate/rank system criticality; project matrix not found in selected pages.</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>MS pp.20,26,31,34,37</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="170" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14" ht="170" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>NC</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>North Carolina / NCDOT</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Asset / vulnerable area / STIP project level, not TAZ</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Multicriteria point matrix using Criticality Score + Exposure Score + Sensitivity Score. Lowest possible = 3 points; highest possible = 12 points. Only assets/projects on Criticality Map and exposed to selected hazards are scored.</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Criticality Score from NCDOT Criticality Map; details not fully in extracted pages. Criticality is one of three point components in the 3-12 scoring matrix.</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Exposure: inland flooding from RIT return intervals (10/25/50/100/500-year), coastal impacts from CRIS/probabilistic SLR, geotechnical from GAM. Sensitivity: roadway IRI &lt;95 good=L, 95-170 fair=M, &gt;170 poor=H; bridges use NBI scour/substructure/channel protection matrices; culverts use NBI Item 62 condition 7-9=L, 5-6=M, 0-4=H; past US-74 washout areas assigned High sensitivity.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Vulnerable areas and STIP projects on Criticality Map and exposed to hazards are ranked by the 3-12 point score.</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>NC pp.49,51-53</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="170" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="15" ht="170" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>NM</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>New Mexico / NMDOT</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Highway segment / hotspot / project-corridor level, not TAZ</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Resilience Risk A-D matrix from Exposure x Sensitivity x Criticality. A=Low, B=Medium, C=High, D=Very High. Exposure/sensitivity/criticality ratings: High=75-100th percentile, Medium=50-74.9th, Low=0-49.9th. Low criticality matrix: high exposure always B; medium exposure A/B/B; low exposure A/A/B. Medium criticality matrix: high exposure B/C/C; medium A/B/C; low A/A/B. High criticality matrix: high exposure C/D/D; medium B/C/D; low B/B/C.</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Criticality converted to High/Medium/Low by percentile; any road/structure on freight network automatically High criticality.</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Exposure, sensitivity, criticality are combined into A-D resilience risk. Only assets with some exposure to at least one hazard are scored.</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Hotspots: adjusted exposure for future wildfire/flood/drought, capped at +/-25%; adjusted risk = adjusted exposure x sensitivity x criticality. High/very-high adjacent segments aggregated into corridors; hotspots ranked by length-weighted average adjusted risk.</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>NM pp.30-32,37</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="170" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16" ht="170" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>OH</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Ohio / ODOT</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Asset level rolled up to corridor/district/state, not TAZ</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Annualized risk-cost model. Risk value = average annual cost of risk from threat likelihood/closure probability and consequences. Consequence cost = owner repair/replacement cost + user disruption/detour cost. Example: flooding damage likelihood = flood likelihood x damage likelihood. Landslide likelihood by susceptibility zone; rockfall likelihood by inventory tier.</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Criticality is embedded in user cost, detour length, staff input on critical sites, and potential future valuation of critical services. No separate point matrix found.</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Vulnerability assessment covers roads/bridges in/near 100-year floodplain for flooding, landslides, rockfalls. Inputs include closure likelihood, damage duration, repair/replacement assumptions, pavement/bridge condition, landslide susceptibility/history, rockfall inventory.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>Priority list developed from risk-based vulnerability assessment results plus district/headquarters input; natural infrastructure/cut sheets for high-vulnerability sites.</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>OH pp.14,16,27,38,51-52</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="170" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17" ht="170" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>OR</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Oregon / ODOT</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Corridor / highway segment level, not TAZ</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Quantitative risk matrix: exposure score 1-5 and consequence score 1-5 averaged into risk score 1.0-5.0. Matrix values: if exposure/consequence are 1/1 =&gt; 1.0; 5/5 =&gt; 5.0; each one-point increase in either dimension adds 0.5. Scores classified by Jenks natural breaks into Low, Medium, High, Very High.</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Consequence measures: functional classification, traffic flow AADT, truck flow AADT. Roadway functional class and AADT indicator scores averaged with equal weights for final consequences score.</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Exposure to nine hazards scored 1-5: extreme temperature, freeze/thaw, extreme precipitation, snowfall, inland flooding, landslides, wildfire, sea level rise/storm surge, coastal erosion.</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Resilience Corridors tiered by future climate, historical hazard events, social disparity status, asset condition, and travel disruption potential; ODOT priority corridors with high truck/traffic flows preferred.</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>OR pp.58,71,78</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="170" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18" ht="170" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>RI</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Rhode Island / RIDOT</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Asset level + criticality/risk map level, not TAZ</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Risk assessment incorporates asset vulnerability with likelihood/probability and consequences/impacts of sea-level rise, storm surge, and inland flooding. TAMP uses likelihood x impact matrix; RIP maps criticality/risk by 2035/2050/2100 and checks acceptable level of change.</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Criticality Score = Usage &amp; Operational Importance 60% + Socioeconomic Importance 20% + Health &amp; Safety Importance 20%. Scores classified High/Medium/Low by percentile.</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>FHWA VAST vulnerability = exposure + sensitivity + adaptive capacity by asset class. Sensitivity example: pavement structural health index 90-100=1, 80-89=2, 70-79=3, 0-69=4. Adaptive capacity examples: low network density scores 4, high density scores 1; downstream stormwater pipes score 4; STU treatment depth 0-2.7 inches scores 4, &gt;7.3 scores 1.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>Need/timeline determined by whether and when risk meets/exceeds acceptable change on criticality/risk matrix maps; project lists and STIP opportunities reviewed.</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>RI pp.39,44,51,57-58,79,167</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="170" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19" ht="170" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Texas / TxDOT</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Asset level, not TAZ</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Relative vulnerability categories minimal-to-high. Vulnerability = exposure + sensitivity. No numeric risk matrix/formula found in extracted main STRP text.</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Evacuation route status used to prioritize assets for strategy development. Performance measures track critical assets damaged multiple times, alternate routes, evacuation route condition. No numeric criticality matrix found.</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Exposure = geospatial overlay of assets with disruptors. Sensitivity = degree to which asset is damaged after exposure. Results reported as high vulnerability counts by asset type/district/disruptor.</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>Resilience strategies intended for standard UTP/project selection and funding; cost-benefit analysis may compare resilience investment cost with future disruptor damages for high-cost strategies.</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>TX pp.57-61,82,85</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="170" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20" ht="170" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>UT</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Utah / UDOT</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Asset segment + candidate project level, not TAZ</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Resilience risk combines normalized exposure score and normalized criticality score. Both use same scale/max and contribute equally. Final risk categories Low to Very High using Jenks natural breaks.</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>Criticality criteria normalized 1-4: system redundancy, AADT, truck AADT, disadvantaged community index, proximity to community assets, transit/bike service. All criteria contribute equally and are summed to criticality score.</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>No separate sensitivity/adaptive capacity component in the extracted UDOT risk equation; asset resilience risk is exposure + criticality.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Candidate project risk assigned two ways: maximum overlapping asset-segment risk and length-weighted average of segment risk. Length-weighted average is basis for prioritized list. Project efficacy score normalized 1-100. Combined score = (candidate project resilience risk + normalized project efficacy score) / 2, equal weights.</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>UT pp.52,56,59-60</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="170" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21" ht="170" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>VA</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Virginia / VDOT</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Asset/infrastructure level planned, not TAZ</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Framework planned, no final matrix. Overall vulnerability will be calculated by assigning weights/percentages to exposure, sensitivity, and criticality.</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>Planned criteria: AADT, roadway designation, redundancy, primary evacuation route, important infrastructure. Weights not finalized.</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Planned elements: exposure to SLR/storm surge/inland flooding and other hazards; sensitivity based on asset condition; criticality. Overall vulnerability = weighted combination of those three elements, but weights not published.</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>Resilience measures can be evaluated through multi-criteria analysis. Steering Committee selects criteria, weights, and ratings; can eliminate measures that do not score well on important criteria. Cost-effectiveness analysis also used.</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>VA pp.25-26,48,55</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="170" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>VT</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Vermont / VTrans</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Project screening level, not TAZ</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Draft screening only. Yes/No flags summed: Highly Vulnerable Location Yes=1; Highly Critical Location Yes=1; Project In Design Yes=1; Ready To Build Yes=1. No full risk matrix found.</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Draft screening asks whether project backs up/increases redundancy for Functional Class 1, 2, and 3 roads, transit, or rail; and whether it improves freight access. Highly Critical Location flag Yes=1.</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>Draft screening asks if project makes a high-risk or documented repeat damage location less likely to be damaged. Highly Vulnerable Location flag Yes=1.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>Draft prioritization scan uses TRPT and Capital Program contents; likely coordinated with VPSP2; yes flags summed for priority scan.</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>VT pp.2-4,9-10</t>
         </is>
@@ -3384,5 +3586,8 @@
   </sheetData>
   <autoFilter ref="A1:H21"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>